<commit_message>
#110 eSpark ,PCBWay ,LCSC BOM Updated
</commit_message>
<xml_diff>
--- a/Deliverables/BOM/LCSC_BOM-v2.1.xlsx
+++ b/Deliverables/BOM/LCSC_BOM-v2.1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\Melih-SoundSensor\Deliverables\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C954E06A-EBF0-4AF8-BCFF-0C5EED4B67D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AB49EF9-8F49-489D-B786-668F370BA2DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="5 Boards" sheetId="5" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="44">
   <si>
     <t>#</t>
   </si>
@@ -149,9 +149,6 @@
     <t>C390772</t>
   </si>
   <si>
-    <t>MOQ (20 Boards)</t>
-  </si>
-  <si>
     <t>MOQ (1K Boards)</t>
   </si>
   <si>
@@ -165,6 +162,12 @@
   </si>
   <si>
     <t>MOQ (5 Boards)</t>
+  </si>
+  <si>
+    <t>C2168289</t>
+  </si>
+  <si>
+    <t>C113030</t>
   </si>
 </sst>
 </file>
@@ -236,7 +239,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -313,11 +316,24 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -350,6 +366,12 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -654,121 +676,121 @@
         <v>2</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="11">
+      <c r="A2" s="2">
         <v>1</v>
       </c>
       <c r="B2" s="5" t="s">
         <v>3</v>
       </c>
       <c r="C2" s="5">
-        <v>120</v>
+        <v>60</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="11">
+      <c r="A3" s="2">
         <v>2</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="5">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="2">
+        <v>3</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="2">
         <v>4</v>
       </c>
-      <c r="C3" s="4">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="11">
-        <v>3</v>
-      </c>
-      <c r="B4" s="5" t="s">
+      <c r="B5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="5">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="2">
         <v>5</v>
       </c>
-      <c r="C4" s="5">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="11">
-        <v>4</v>
-      </c>
-      <c r="B5" s="4" t="s">
+      <c r="B6" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C6" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="2">
         <v>6</v>
       </c>
-      <c r="C5" s="4">
+      <c r="B7" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C7" s="5">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="2">
+        <v>7</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="C8" s="5">
         <v>100</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="11">
-        <v>5</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C6" s="5">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="11">
-        <v>6</v>
-      </c>
-      <c r="B7" s="4" t="s">
+    <row r="9" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="2">
         <v>8</v>
       </c>
-      <c r="C7" s="4">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="11">
-        <v>7</v>
-      </c>
-      <c r="B8" s="5" t="s">
+      <c r="B9" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C9" s="5">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="2">
         <v>9</v>
       </c>
-      <c r="C8" s="5">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="11">
-        <v>8</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="C9" s="4">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="11">
-        <v>9</v>
-      </c>
       <c r="B10" s="5" t="s">
-        <v>11</v>
+        <v>42</v>
       </c>
       <c r="C10" s="5">
         <v>60</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="11">
+      <c r="A11" s="2">
         <v>10</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="B11" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="C11" s="4">
+      <c r="C11" s="5">
         <v>100</v>
       </c>
     </row>
     <row r="12" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="11">
+      <c r="A12" s="2">
         <v>11</v>
       </c>
       <c r="B12" s="5" t="s">
@@ -779,244 +801,244 @@
       </c>
     </row>
     <row r="13" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="11">
+      <c r="A13" s="2">
         <v>12</v>
       </c>
-      <c r="B13" s="4" t="s">
+      <c r="B13" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="C13" s="4">
+      <c r="C13" s="5">
         <v>100</v>
       </c>
     </row>
     <row r="14" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="11">
+      <c r="A14" s="2">
         <v>13</v>
       </c>
       <c r="B14" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C14" s="5">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="2">
+        <v>14</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C15" s="5">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="2">
         <v>15</v>
       </c>
-      <c r="C14" s="5">
+      <c r="B16" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="C16" s="5">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="2">
+        <v>16</v>
+      </c>
+      <c r="B17" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="C17" s="5">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="2">
+        <v>17</v>
+      </c>
+      <c r="B18" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C18" s="5">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="2">
+        <v>18</v>
+      </c>
+      <c r="B19" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="C19" s="5">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="2">
+        <v>19</v>
+      </c>
+      <c r="B20" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C20" s="5">
         <v>100</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="11">
-        <v>14</v>
-      </c>
-      <c r="B15" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="C15" s="4">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="11">
-        <v>15</v>
-      </c>
-      <c r="B16" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="C16" s="4">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="11">
-        <v>16</v>
-      </c>
-      <c r="B17" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="C17" s="5">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="11">
-        <v>17</v>
-      </c>
-      <c r="B18" s="4" t="s">
+    <row r="21" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="2">
         <v>20</v>
       </c>
-      <c r="C18" s="4">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="11">
-        <v>18</v>
-      </c>
-      <c r="B19" s="5" t="s">
+      <c r="B21" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="C21" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="2">
         <v>21</v>
       </c>
-      <c r="C19" s="5">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="11">
-        <v>19</v>
-      </c>
-      <c r="B20" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="C20" s="4">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="11">
-        <v>20</v>
-      </c>
-      <c r="B21" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="C21" s="4">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="11">
-        <v>21</v>
-      </c>
       <c r="B22" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C22" s="5">
         <v>100</v>
       </c>
     </row>
     <row r="23" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="11">
+      <c r="A23" s="2">
         <v>22</v>
       </c>
-      <c r="B23" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="C23" s="4">
+      <c r="B23" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="C23" s="5">
         <v>100</v>
       </c>
     </row>
     <row r="24" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="11">
+      <c r="A24" s="2">
         <v>23</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C24" s="5">
         <v>100</v>
       </c>
     </row>
     <row r="25" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="11">
+      <c r="A25" s="2">
         <v>24</v>
       </c>
-      <c r="B25" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="C25" s="4">
+      <c r="B25" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="C25" s="5">
         <v>100</v>
       </c>
     </row>
     <row r="26" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="11">
+      <c r="A26" s="2">
         <v>25</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C26" s="5">
         <v>100</v>
       </c>
     </row>
     <row r="27" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="11">
+      <c r="A27" s="2">
         <v>26</v>
       </c>
-      <c r="B27" s="4" t="s">
+      <c r="B27" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="C27" s="5">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="2">
+        <v>27</v>
+      </c>
+      <c r="B28" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="C28" s="5">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="2">
+        <v>28</v>
+      </c>
+      <c r="B29" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="C29" s="5">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="2">
         <v>29</v>
       </c>
-      <c r="C27" s="4">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="11">
-        <v>27</v>
-      </c>
-      <c r="B28" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="C28" s="4">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="11">
-        <v>28</v>
-      </c>
-      <c r="B29" s="5" t="s">
+      <c r="B30" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="C30" s="5">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="2">
         <v>30</v>
       </c>
-      <c r="C29" s="5">
+      <c r="B31" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C31" s="5">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A32" s="2">
+        <v>31</v>
+      </c>
+      <c r="B32" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="C32" s="5">
         <v>6</v>
       </c>
     </row>
-    <row r="30" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="11">
-        <v>29</v>
-      </c>
-      <c r="B30" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="C30" s="4">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="11">
-        <v>30</v>
-      </c>
-      <c r="B31" s="5" t="s">
+    <row r="33" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A33" s="2">
         <v>32</v>
       </c>
-      <c r="C31" s="5">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="11">
-        <v>31</v>
-      </c>
-      <c r="B32" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="C32" s="5">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="11">
-        <v>32</v>
-      </c>
       <c r="B33" s="5" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C33" s="5">
-        <v>6</v>
+        <v>15</v>
       </c>
     </row>
     <row r="34" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="11">
         <v>33</v>
       </c>
-      <c r="B34" s="8" t="s">
+      <c r="B34" s="13" t="s">
         <v>36</v>
       </c>
-      <c r="C34" s="8">
+      <c r="C34" s="13">
         <v>15</v>
       </c>
     </row>
@@ -1027,7 +1049,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B9C0EAC8-2749-4D8B-AD6B-98E76B44D0B5}">
-  <dimension ref="A1:C35"/>
+  <dimension ref="A1:C34"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="3" bestFit="1" customWidth="1"/>
@@ -1037,378 +1059,169 @@
   <sheetData>
     <row r="1" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="10" t="s">
-        <v>2</v>
-      </c>
-      <c r="C2" s="10" t="s">
-        <v>37</v>
-      </c>
+      <c r="A2" s="3"/>
+      <c r="B2" s="10"/>
+      <c r="C2" s="10"/>
     </row>
     <row r="3" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="2">
-        <v>1</v>
-      </c>
-      <c r="B3" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="C3" s="5">
-        <v>450</v>
-      </c>
+      <c r="A3" s="2"/>
+      <c r="B3" s="5"/>
+      <c r="C3" s="5"/>
     </row>
     <row r="4" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="2">
-        <v>2</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="C4" s="4">
-        <v>40</v>
-      </c>
+      <c r="A4" s="2"/>
+      <c r="B4" s="5"/>
+      <c r="C4" s="5"/>
     </row>
     <row r="5" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="2">
-        <v>3</v>
-      </c>
-      <c r="B5" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="C5" s="5">
-        <v>900</v>
-      </c>
+      <c r="A5" s="2"/>
+      <c r="B5" s="5"/>
+      <c r="C5" s="5"/>
     </row>
     <row r="6" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="2">
-        <v>4</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="C6" s="4">
-        <v>300</v>
-      </c>
+      <c r="A6" s="2"/>
+      <c r="B6" s="5"/>
+      <c r="C6" s="5"/>
     </row>
     <row r="7" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="2">
-        <v>5</v>
-      </c>
-      <c r="B7" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C7" s="5">
-        <v>45</v>
-      </c>
+      <c r="A7" s="2"/>
+      <c r="B7" s="5"/>
+      <c r="C7" s="5"/>
     </row>
     <row r="8" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="2">
-        <v>6</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C8" s="4">
-        <v>400</v>
-      </c>
+      <c r="A8" s="2"/>
+      <c r="B8" s="5"/>
+      <c r="C8" s="5"/>
     </row>
     <row r="9" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="2">
-        <v>7</v>
-      </c>
-      <c r="B9" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="C9" s="5">
-        <v>30</v>
-      </c>
+      <c r="A9" s="2"/>
+      <c r="B9" s="5"/>
+      <c r="C9" s="5"/>
     </row>
     <row r="10" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="2">
-        <v>8</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="C10" s="4">
-        <v>200</v>
-      </c>
+      <c r="A10" s="2"/>
+      <c r="B10" s="5"/>
+      <c r="C10" s="5"/>
     </row>
     <row r="11" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="2">
-        <v>9</v>
-      </c>
-      <c r="B11" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="C11" s="5">
-        <v>230</v>
-      </c>
+      <c r="A11" s="2"/>
+      <c r="B11" s="5"/>
+      <c r="C11" s="5"/>
     </row>
     <row r="12" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="2">
-        <v>10</v>
-      </c>
-      <c r="B12" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="C12" s="4">
-        <v>100</v>
-      </c>
+      <c r="A12" s="2"/>
+      <c r="B12" s="5"/>
+      <c r="C12" s="5"/>
     </row>
     <row r="13" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="2">
-        <v>11</v>
-      </c>
-      <c r="B13" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="C13" s="5">
-        <v>100</v>
-      </c>
+      <c r="A13" s="2"/>
+      <c r="B13" s="5"/>
+      <c r="C13" s="5"/>
     </row>
     <row r="14" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="2">
-        <v>12</v>
-      </c>
-      <c r="B14" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="C14" s="4">
-        <v>200</v>
-      </c>
+      <c r="A14" s="2"/>
+      <c r="B14" s="5"/>
+      <c r="C14" s="5"/>
     </row>
     <row r="15" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="2">
-        <v>13</v>
-      </c>
-      <c r="B15" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="C15" s="5">
-        <v>200</v>
-      </c>
+      <c r="A15" s="2"/>
+      <c r="B15" s="5"/>
+      <c r="C15" s="5"/>
     </row>
     <row r="16" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="2">
-        <v>14</v>
-      </c>
-      <c r="B16" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="C16" s="4">
-        <v>170</v>
-      </c>
+      <c r="A16" s="2"/>
+      <c r="B16" s="5"/>
+      <c r="C16" s="5"/>
     </row>
     <row r="17" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="2">
-        <v>15</v>
-      </c>
-      <c r="B17" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="C17" s="4">
-        <v>30</v>
-      </c>
+      <c r="A17" s="2"/>
+      <c r="B17" s="12"/>
+      <c r="C17" s="5"/>
     </row>
     <row r="18" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="2">
-        <v>16</v>
-      </c>
-      <c r="B18" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="C18" s="5">
-        <v>30</v>
-      </c>
+      <c r="A18" s="2"/>
+      <c r="B18" s="5"/>
+      <c r="C18" s="5"/>
     </row>
     <row r="19" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="2">
-        <v>17</v>
-      </c>
-      <c r="B19" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="C19" s="4">
-        <v>40</v>
-      </c>
+      <c r="A19" s="2"/>
+      <c r="B19" s="5"/>
+      <c r="C19" s="5"/>
     </row>
     <row r="20" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="2">
-        <v>18</v>
-      </c>
-      <c r="B20" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="C20" s="5">
-        <v>30</v>
-      </c>
+      <c r="A20" s="2"/>
+      <c r="B20" s="5"/>
+      <c r="C20" s="5"/>
     </row>
     <row r="21" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="2">
-        <v>19</v>
-      </c>
-      <c r="B21" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="C21" s="4">
-        <v>40</v>
-      </c>
+      <c r="A21" s="2"/>
+      <c r="B21" s="5"/>
+      <c r="C21" s="5"/>
     </row>
     <row r="22" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="2">
-        <v>20</v>
-      </c>
-      <c r="B22" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="C22" s="7">
-        <v>100</v>
-      </c>
+      <c r="A22" s="2"/>
+      <c r="B22" s="5"/>
+      <c r="C22" s="5"/>
     </row>
     <row r="23" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="2">
-        <v>21</v>
-      </c>
-      <c r="B23" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="C23" s="5">
-        <v>200</v>
-      </c>
+      <c r="A23" s="2"/>
+      <c r="B23" s="5"/>
+      <c r="C23" s="5"/>
     </row>
     <row r="24" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="2">
-        <v>22</v>
-      </c>
-      <c r="B24" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="C24" s="4">
-        <v>100</v>
-      </c>
+      <c r="A24" s="2"/>
+      <c r="B24" s="5"/>
+      <c r="C24" s="5"/>
     </row>
     <row r="25" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="2">
-        <v>23</v>
-      </c>
-      <c r="B25" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="C25" s="5">
-        <v>300</v>
-      </c>
+      <c r="A25" s="2"/>
+      <c r="B25" s="5"/>
+      <c r="C25" s="5"/>
     </row>
     <row r="26" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="2">
-        <v>24</v>
-      </c>
-      <c r="B26" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="C26" s="4">
-        <v>100</v>
-      </c>
+      <c r="A26" s="2"/>
+      <c r="B26" s="5"/>
+      <c r="C26" s="5"/>
     </row>
     <row r="27" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="2">
-        <v>25</v>
-      </c>
-      <c r="B27" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="C27" s="5">
-        <v>400</v>
-      </c>
+      <c r="A27" s="2"/>
+      <c r="B27" s="5"/>
+      <c r="C27" s="5"/>
     </row>
     <row r="28" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="2">
-        <v>26</v>
-      </c>
-      <c r="B28" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="C28" s="4">
-        <v>100</v>
-      </c>
+      <c r="A28" s="2"/>
+      <c r="B28" s="5"/>
+      <c r="C28" s="5"/>
     </row>
     <row r="29" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="2">
-        <v>27</v>
-      </c>
-      <c r="B29" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="C29" s="4">
-        <v>30</v>
-      </c>
+      <c r="A29" s="2"/>
+      <c r="B29" s="5"/>
+      <c r="C29" s="5"/>
     </row>
     <row r="30" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="2">
-        <v>28</v>
-      </c>
-      <c r="B30" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="C30" s="5">
-        <v>22</v>
-      </c>
+      <c r="A30" s="2"/>
+      <c r="B30" s="5"/>
+      <c r="C30" s="5"/>
     </row>
     <row r="31" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="2">
-        <v>29</v>
-      </c>
-      <c r="B31" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="C31" s="4">
-        <v>165</v>
-      </c>
+      <c r="A31" s="2"/>
+      <c r="B31" s="5"/>
+      <c r="C31" s="5"/>
     </row>
     <row r="32" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="2">
-        <v>30</v>
-      </c>
-      <c r="B32" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="C32" s="5">
-        <v>22</v>
-      </c>
+      <c r="A32" s="2"/>
+      <c r="B32" s="5"/>
+      <c r="C32" s="5"/>
     </row>
     <row r="33" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="2">
-        <v>31</v>
-      </c>
-      <c r="B33" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="C33" s="5">
-        <v>42</v>
-      </c>
+      <c r="A33" s="2"/>
+      <c r="B33" s="5"/>
+      <c r="C33" s="5"/>
     </row>
     <row r="34" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="2">
-        <v>32</v>
-      </c>
-      <c r="B34" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="C34" s="5">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="2">
-        <v>33</v>
-      </c>
-      <c r="B35" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="C35" s="4">
-        <v>45</v>
-      </c>
+      <c r="A34" s="2"/>
+      <c r="B34" s="5"/>
+      <c r="C34" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1433,7 +1246,7 @@
         <v>2</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1921,7 +1734,7 @@
         <v>2</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">

</xml_diff>